<commit_message>
Update Student Exam Page
</commit_message>
<xml_diff>
--- a/OEMS - 20225/Template/C Programming Import Template.xlsx
+++ b/OEMS - 20225/Template/C Programming Import Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2. Personal Workspace\05 Study Resources\CUG\Final Thesis\OEMS - 20225\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28912476-AC60-48AE-A183-35A87FB39C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{521613DA-CB5E-46C9-8861-26738A436129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{13CFBFC4-CC69-4375-817A-07D88E34A5F9}"/>
   </bookViews>
@@ -678,9 +678,14 @@
   <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
+    <col min="1" max="1" width="24.734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.05078125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.89453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.68359375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.3125" customWidth="1"/>
+    <col min="8" max="8" width="7.89453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.41796875" customWidth="1"/>
+    <col min="10" max="10" width="17.68359375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
@@ -1035,7 +1040,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="2" t="s">
         <v>58</v>
       </c>
@@ -1067,7 +1072,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="144" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" ht="72" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="2" t="s">
         <v>61</v>
       </c>
@@ -1099,7 +1104,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="2" t="s">
         <v>66</v>
       </c>
@@ -1131,7 +1136,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="2" t="s">
         <v>69</v>
       </c>
@@ -1163,7 +1168,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="2" t="s">
         <v>70</v>
       </c>
@@ -1195,7 +1200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="129.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="2" t="s">
         <v>72</v>
       </c>
@@ -1227,7 +1232,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="2" t="s">
         <v>77</v>
       </c>
@@ -1259,7 +1264,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="2" t="s">
         <v>80</v>
       </c>
@@ -1291,7 +1296,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="129.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="2" t="s">
         <v>85</v>
       </c>
@@ -1323,7 +1328,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="2" t="s">
         <v>88</v>
       </c>

</xml_diff>